<commit_message>
feat(analyses): TP M3-2 v3 — fusion v2 et distinction AIPD / analyse de risques
Reprend la v2 du collegue (ligne 6 cotee sur l'echelle sante, ligne 9
injection de fausses donnees, ligne 7 reclassee technique, ligne 10
materiovigilance, colonne etat des mesures) et repond a la remarque de
l'intervenant : section dediee sur l'analyse d'impact RGPD, criteres de
la liste CNIL, acces, durees de conservation, information des residents.
Ajoute le fait verifie du pont Mosquitto vers broker.hivemq.com public.
</commit_message>
<xml_diff>
--- a/analyses/m3/analyse_risques_eq05.xlsx
+++ b/analyses/m3/analyse_risques_eq05.xlsx
@@ -1415,7 +1415,7 @@
       </c>
       <c r="R9" s="19" t="inlineStr">
         <is>
-          <t>Lien M2 : calcul d'autonomie du TP M2-4, à confirmer par la mesure au projet 1. Grave reste grave : au mieux « moyen ». Bénéfice : les chutes de nuit sont signalées en minutes, pas découvertes à la ronde.</t>
+          <t>Lien M2 : l'autonomie de 7 jours est un OBJECTIF de conception : le TP M2-4 n'est pas dans le dépôt, le chiffre n'est donc pas encore mesuré (à mesurer au projet 1 ; si l'autonomie réelle est plus courte, la probabilité résiduelle remonte). Grave reste grave : au mieux « moyen ». Bénéfice : les chutes de nuit sont signalées en minutes, pas découvertes à la ronde.</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="K10" s="21" t="inlineStr">
         <is>
-          <t>Règle à trois temps du TP M2-2 (chute libre → impact → immobilité) réglée pour privilégier le rappel, complétée par une détection d'immobilité prolongée au sol et par les capteurs de présence de la chambre (fusion de sources)</t>
+          <t>Règle à trois temps du TP M2-2 réglée pour privilégier le rappel, complétée par une détection d'immobilité prolongée au sol ; ajout d'une détection indépendante du bracelet : capteur de présence au sol dans la chambre (radar ou tapis), actif la nuit (fusion de sources : une chute ratée par le bracelet peut être vue par la chambre)</t>
         </is>
       </c>
       <c r="L10" s="21" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="R10" s="21" t="inlineStr">
         <is>
-          <t>Lien M2 : règle à trois temps du TP M2-2 (précision 1,00 sur le jeu de secours, mais une personne âgée ne tombe pas comme un téléphone : à revalider sur des chutes humaines). La gravité ne descend pas : bénéfice = une chute signalée en minutes au lieu d'être découverte à la ronde suivante.</t>
+          <t>Lien M2 : la règle à trois temps n'a été testée que sur le jeu de secours SYNTHÉTIQUE (chutes de téléphone) ; la conclusion du TP M2-2 dit elle-même qu'elle rate le profil d'une chute humaine. Le bracelet seul ne justifie donc PAS « rare » : c'est le capteur de chambre indépendant qui fait descendre la probabilité. Cotation « rare » conditionnée à une validation sur des chutes humaines au projet 1 ; sans elle, le risque reste à 3 × 2 = 6 (élevé) et le système ne peut pas remplacer les rondes. Bénéfice : une chute signalée en minutes au lieu d'être découverte à la ronde suivante.</t>
         </is>
       </c>
     </row>
@@ -1742,12 +1742,12 @@
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>Données de santé interceptées sur le réseau</t>
+          <t>Données de santé interceptées sur le réseau (atteinte à la vie privée)</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>MQTT publié en clair et Bluetooth non appairé → un tiers présent sur le réseau de l'établissement écoute le trafic → constantes, déplacements et horaires des résidents captés</t>
+          <t>MQTT publié en clair (port 1883, sans TLS : état actuel du dépôt) et Bluetooth non appairé → un tiers présent sur le réseau de l'établissement écoute le trafic → constantes, déplacements et horaires des résidents captés</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="F14" s="21" t="inlineStr">
         <is>
-          <t>Atteinte à la vie privée (donnée de santé, RGPD art. 9) et repérage des absences ; pas d'atteinte physique directe, mais perte de confiance et signalement CNIL</t>
+          <t>Atteinte à la vie privée (donnée de santé, RGPD art. 9), repérage des absences ; pas d'atteinte physique directe ni de soins nécessaires</t>
         </is>
       </c>
       <c r="G14" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="22" t="n">
         <v>2</v>
@@ -1790,7 +1790,7 @@
         </is>
       </c>
       <c r="N14" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="22" t="n">
         <v>1</v>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="R14" s="21" t="inlineStr">
         <is>
-          <t>Lien M2 : addendum sécurité (TLS 8883, certificat par objet, comptes séparés). Cadre : IEC 81001-5-1 et guide MDCG 2019-16 sur la cybersécurité des dispositifs médicaux. Risque résiduel faible, accepté.</t>
+          <t>Gravité cotée 1 : l'échelle du cours mesure l'atteinte à la SANTÉ (« Modérée » = soins nécessaires, ce qui n'est pas le cas ici). Ce score faible ne veut pas dire que le risque est négligeable : il relève aussi du RGPD (AIPD) et de l'IEC 81001-5-1 / MDCG 2019-16, traités hors de cette matrice. MESURES À METTRE EN ŒUVRE : le dépôt est aujourd'hui en 1883 sans TLS avec allow_anonymous true (docs/contrat_mqtt.md) ; la cotation résiduelle ne vaut qu'une fois TLS 8883 et les certificats en place. Fait vérifié dans le dépôt : le pont Mosquitto relaie vitals/resident/+, motion/resident/+ et alerts/new vers broker.hivemq.com, broker PUBLIC en 1883 anonyme (mosquitto/config/mosquitto.conf). Données fictives aujourd'hui ; ce pont doit disparaître avant toute donnée réelle, et il est à décrire tel quel dans l'AIPD.</t>
         </is>
       </c>
     </row>
@@ -1815,17 +1815,17 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>Cybersécurité</t>
+          <t>Technique</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
         <is>
-          <t>Surveillance interrompue : broker saturé, réseau coupé ou brouillé</t>
+          <t>Surveillance interrompue : broker saturé ou réseau coupé</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>Saturation du broker, panne Wi-Fi ou brouillage → plus aucun message ne remonte → le tableau de bord continue d'afficher les dernières valeurs connues → les soignants croient la surveillance active</t>
+          <t>Saturation du broker ou panne Wi-Fi → plus aucun message ne remonte → le tableau de bord continue d'afficher les dernières valeurs connues → les soignants croient la surveillance active</t>
         </is>
       </c>
       <c r="E15" s="21" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="R15" s="21" t="inlineStr">
         <is>
-          <t>Aucune donnée périmée affichée comme fraîche : c'est la règle « mesure indisponible » du M2 appliquée au transport. Gravité irréductible ; bénéfice : la panne devient visible en minutes au lieu d'être découverte après coup.</t>
+          <t>Reclassé en « Technique » : une panne ou une saturation n'est pas une attaque (l'attaque volontaire est traitée ligne 9). Aucune donnée périmée affichée comme fraîche : c'est la règle « mesure indisponible » du M2 appliquée au transport. Gravité irréductible ; bénéfice : la panne devient visible en minutes au lieu d'être découverte après coup. À distinguer de l'AIPD : ici le dommage est l'absence de secours, pas la fuite de données.</t>
         </is>
       </c>
     </row>
@@ -1969,13 +1969,37 @@
       <c r="A17" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="21" t="n"/>
-      <c r="G17" s="22" t="n"/>
-      <c r="H17" s="22" t="n"/>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Cybersécurité</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>Fausses données injectées : un client non autorisé publie sur le broker</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>Broker accessible sans authentification (allow_anonymous true, port 1883 : état actuel du dépôt) → un client non autorisé publie de fausses constantes « normales », ou brouille / sature le canal, sur les topics d'un résident → la vraie chute est masquée ou noyée</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>La résidente est au sol, le tableau de bord affiche des constantes normales</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>Chute ou malaise non pris en charge : attente prolongée au sol, aggravation, hospitalisation</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" s="22" t="n">
+        <v>2</v>
+      </c>
       <c r="I17" s="13">
         <f>IF(OR(G17="",H17=""),"",G17*H17)</f>
         <v/>
@@ -1984,11 +2008,27 @@
         <f>IF(I17="","",IF(I17&gt;='Échelles'!$C$15,"Élevé : inacceptable",IF(I17&gt;='Échelles'!$C$14,"Moyen : à réduire","Faible : acceptable")))</f>
         <v/>
       </c>
-      <c r="K17" s="21" t="n"/>
-      <c r="L17" s="21" t="n"/>
-      <c r="M17" s="21" t="n"/>
-      <c r="N17" s="22" t="n"/>
-      <c r="O17" s="22" t="n"/>
+      <c r="K17" s="21" t="inlineStr">
+        <is>
+          <t>Authentification mutuelle TLS sur le port 8883 avec un certificat par objet (addendum sécurité M2) ; allow_anonymous false ; ACL par topic : chaque objet ne publie que sur son propre topic, seul le backend publie les alertes ; numéro de séquence et horodatage dans chaque message (anti-rejeu)</t>
+        </is>
+      </c>
+      <c r="L17" s="21" t="inlineStr">
+        <is>
+          <t>Alerte sécurité au poste de soins sur connexion refusée, saut de séquence ou deux sources pour un même capteur ; journalisation des connexions ; bascule en « système dégradé » (comme ligne 7) si l'intégrité est douteuse</t>
+        </is>
+      </c>
+      <c r="M17" s="21" t="inlineStr">
+        <is>
+          <t>Procédure de gestion des certificats (émission, révocation d'un bracelet perdu) ; plan de réponse à incident ; formation du personnel : signaler toute alerte ou valeur incohérente</t>
+        </is>
+      </c>
+      <c r="N17" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="22" t="n">
+        <v>1</v>
+      </c>
       <c r="P17" s="13">
         <f>IF(OR(N17="",O17=""),"",N17*O17)</f>
         <v/>
@@ -1997,19 +2037,47 @@
         <f>IF(P17="","",IF(P17&gt;='Échelles'!$C$15,"Élevé : inacceptable",IF(P17&gt;='Échelles'!$C$14,"Moyen : à réduire","Faible : acceptable")))</f>
         <v/>
       </c>
-      <c r="R17" s="21" t="n"/>
+      <c r="R17" s="21" t="inlineStr">
+        <is>
+          <t>Lien M2 : addendum sécurité (TLS 8883, certificat par objet, comptes séparés). Cadre : IEC 81001-5-1, MDCG 2019-16. C'est le vrai danger cyber pour le PATIENT : une attaque qui masque une chute est un risque de santé, pas seulement de données. MESURES À METTRE EN ŒUVRE : tant que le broker reste anonyme en 1883, le risque reste à 3 × 2 = 6 (élevé). Gravité irréductible ; bénéfice : seules les données authentifiées peuvent déclencher ou masquer une alerte.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="B18" s="21" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="21" t="n"/>
-      <c r="G18" s="22" t="n"/>
-      <c r="H18" s="22" t="n"/>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Exemple de matériovigilance (hors projet) : canule du pod Omnipod qui peut se déchirer (rappel de lots ANSM, 3 juin 2026)</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Canule déchirée sous la peau → moins d'insuline délivrée que la dose programmée → le patient ne s'en rend pas compte</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Patient diabétique sous-dosé en insuline sans le savoir</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Hyperglycémie, pouvant aller jusqu'à l'acidocétose et l'hospitalisation</t>
+        </is>
+      </c>
+      <c r="G18" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="22" t="n">
+        <v>2</v>
+      </c>
       <c r="I18" s="13">
         <f>IF(OR(G18="",H18=""),"",G18*H18)</f>
         <v/>
@@ -2018,11 +2086,27 @@
         <f>IF(I18="","",IF(I18&gt;='Échelles'!$C$15,"Élevé : inacceptable",IF(I18&gt;='Échelles'!$C$14,"Moyen : à réduire","Faible : acceptable")))</f>
         <v/>
       </c>
-      <c r="K18" s="21" t="n"/>
-      <c r="L18" s="21" t="n"/>
-      <c r="M18" s="21" t="n"/>
-      <c r="N18" s="22" t="n"/>
-      <c r="O18" s="22" t="n"/>
+      <c r="K18" s="21" t="inlineStr">
+        <is>
+          <t>Correction du procédé de fabrication de la canule ; contrôle renforcé des lots</t>
+        </is>
+      </c>
+      <c r="L18" s="21" t="inlineStr">
+        <is>
+          <t>Rappel des lots concernés ; alerte d'occlusion ou de délivrance anormale ; surveillance glycémique (capteur de glucose) qui signale la dérive</t>
+        </is>
+      </c>
+      <c r="M18" s="21" t="inlineStr">
+        <is>
+          <t>Information de sécurité aux patients et aux soignants ; consigne : surveiller la glycémie et changer le pod en cas de valeurs hautes inexpliquées</t>
+        </is>
+      </c>
+      <c r="N18" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" s="22" t="n">
+        <v>1</v>
+      </c>
       <c r="P18" s="13">
         <f>IF(OR(N18="",O18=""),"",N18*O18)</f>
         <v/>
@@ -2031,7 +2115,11 @@
         <f>IF(P18="","",IF(P18&gt;='Échelles'!$C$15,"Élevé : inacceptable",IF(P18&gt;='Échelles'!$C$14,"Moyen : à réduire","Faible : acceptable")))</f>
         <v/>
       </c>
-      <c r="R18" s="21" t="n"/>
+      <c r="R18" s="21" t="inlineStr">
+        <is>
+          <t>Exemple « pour aller plus loin », hors périmètre de notre projet : à retirer à l'analyse de risques v1 (projet 1). Il montre que l'analyse de risques continue après la vente : un incident remonté (matériovigilance) rouvre le dossier.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">

</xml_diff>